<commit_message>
fix(test): excel append isolation + canonical 4-sheet structural seed
- The committed Inventory_with_Photos.xlsx seed was the accidental 1-sheet
  workbook (the exact drift scripts/seed-inventory-with-photos.mjs warns
  about), so the canonical-sheets assertions failed on fresh clones.
  Regenerated via the seed script: Owners Rent/Buy + Broker Rent/Buy.
- appendToExcelInventory test now appends to a throwaway temp copy instead
  of the resolved master path: the old test mutated the runtime master and
  left a root-level artifact that shadowed the structural seed on every
  later run (getMasterExcelPath prefers the root runtime file).
- Hazard documented at the top of the suite.
- Root vitest: 713/713 green.
</commit_message>
<xml_diff>
--- a/apps/sierra-estates-realty/data/Inventory_with_Photos.xlsx
+++ b/apps/sierra-estates-realty/data/Inventory_with_Photos.xlsx
@@ -535,7 +535,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V2" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +603,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V3" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
   </sheetData>
@@ -615,7 +615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -750,7 +750,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V2" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
     <row r="3">
@@ -818,692 +818,12 @@
         <v>structural-seed</v>
       </c>
       <c r="V3" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>TEST-OWNER-MVEPZOHF</v>
-      </c>
-      <c r="B4" t="str">
-        <v>TEST-OWNER-MVEPZOHF</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D4" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E4" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H4">
-        <v>14500000</v>
-      </c>
-      <c r="I4" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J4">
-        <v>170</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N4" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R4" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S4" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T4" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U4" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V4" t="str">
-        <v>2026-10-19T03:54:04.085Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>TEST-OWNER-MVEPZRV5</v>
-      </c>
-      <c r="B5" t="str">
-        <v>TEST-OWNER-MVEPZRV5</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D5" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E5" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H5">
-        <v>14500000</v>
-      </c>
-      <c r="I5" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J5">
-        <v>170</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N5" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R5" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S5" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T5" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U5" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V5" t="str">
-        <v>2026-10-19T03:54:08.468Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>TEST-OWNER-MVEQ0CYJ</v>
-      </c>
-      <c r="B6" t="str">
-        <v>TEST-OWNER-MVEQ0CYJ</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D6" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E6" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H6">
-        <v>14500000</v>
-      </c>
-      <c r="I6" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J6">
-        <v>170</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>2</v>
-      </c>
-      <c r="M6" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N6" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R6" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S6" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T6" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U6" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V6" t="str">
-        <v>2026-10-19T03:54:35.806Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>TEST-OWNER-MVEQ85DQ</v>
-      </c>
-      <c r="B7" t="str">
-        <v>TEST-OWNER-MVEQ85DQ</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D7" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E7" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H7">
-        <v>14500000</v>
-      </c>
-      <c r="I7" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J7">
-        <v>170</v>
-      </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-      <c r="L7">
-        <v>2</v>
-      </c>
-      <c r="M7" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N7" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O7" t="str">
-        <v/>
-      </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-      <c r="Q7" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R7" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S7" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T7" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U7" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V7" t="str">
-        <v>2026-10-19T04:00:39.232Z</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>TEST-OWNER-MVEQ8SGX</v>
-      </c>
-      <c r="B8" t="str">
-        <v>TEST-OWNER-MVEQ8SGX</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D8" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E8" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H8">
-        <v>14500000</v>
-      </c>
-      <c r="I8" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J8">
-        <v>170</v>
-      </c>
-      <c r="K8">
-        <v>3</v>
-      </c>
-      <c r="L8">
-        <v>2</v>
-      </c>
-      <c r="M8" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N8" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O8" t="str">
-        <v/>
-      </c>
-      <c r="P8" t="str">
-        <v/>
-      </c>
-      <c r="Q8" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R8" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S8" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T8" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U8" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V8" t="str">
-        <v>2026-10-19T04:01:09.155Z</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>TEST-OWNER-MVEQ9LS6</v>
-      </c>
-      <c r="B9" t="str">
-        <v>TEST-OWNER-MVEQ9LS6</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D9" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E9" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H9">
-        <v>14500000</v>
-      </c>
-      <c r="I9" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J9">
-        <v>170</v>
-      </c>
-      <c r="K9">
-        <v>3</v>
-      </c>
-      <c r="L9">
-        <v>2</v>
-      </c>
-      <c r="M9" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N9" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O9" t="str">
-        <v/>
-      </c>
-      <c r="P9" t="str">
-        <v/>
-      </c>
-      <c r="Q9" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R9" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S9" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T9" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U9" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V9" t="str">
-        <v>2026-10-19T04:01:47.145Z</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>TEST-OWNER-MVEQA0E6</v>
-      </c>
-      <c r="B10" t="str">
-        <v>TEST-OWNER-MVEQA0E6</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D10" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E10" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H10">
-        <v>14500000</v>
-      </c>
-      <c r="I10" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J10">
-        <v>170</v>
-      </c>
-      <c r="K10">
-        <v>3</v>
-      </c>
-      <c r="L10">
-        <v>2</v>
-      </c>
-      <c r="M10" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N10" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O10" t="str">
-        <v/>
-      </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-      <c r="Q10" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R10" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S10" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T10" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U10" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V10" t="str">
-        <v>2026-10-19T04:02:06.081Z</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>TEST-OWNER-MVEQAN4P</v>
-      </c>
-      <c r="B11" t="str">
-        <v>TEST-OWNER-MVEQAN4P</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D11" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E11" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H11">
-        <v>14500000</v>
-      </c>
-      <c r="I11" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J11">
-        <v>170</v>
-      </c>
-      <c r="K11">
-        <v>3</v>
-      </c>
-      <c r="L11">
-        <v>2</v>
-      </c>
-      <c r="M11" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N11" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O11" t="str">
-        <v/>
-      </c>
-      <c r="P11" t="str">
-        <v/>
-      </c>
-      <c r="Q11" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R11" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S11" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T11" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U11" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V11" t="str">
-        <v>2026-10-19T04:02:35.547Z</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>TEST-OWNER-MVEQG3MN</v>
-      </c>
-      <c r="B12" t="str">
-        <v>TEST-OWNER-MVEQG3MN</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D12" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E12" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H12">
-        <v>14500000</v>
-      </c>
-      <c r="I12" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J12">
-        <v>170</v>
-      </c>
-      <c r="K12">
-        <v>3</v>
-      </c>
-      <c r="L12">
-        <v>2</v>
-      </c>
-      <c r="M12" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N12" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O12" t="str">
-        <v/>
-      </c>
-      <c r="P12" t="str">
-        <v/>
-      </c>
-      <c r="Q12" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R12" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S12" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T12" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U12" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V12" t="str">
-        <v>2026-10-19T04:06:50.211Z</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>TEST-OWNER-MVEQM170</v>
-      </c>
-      <c r="B13" t="str">
-        <v>TEST-OWNER-MVEQM170</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Mivida</v>
-      </c>
-      <c r="D13" t="str">
-        <v>New Cairo</v>
-      </c>
-      <c r="E13" t="str">
-        <v>5th Settlement</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Apartment</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Sale</v>
-      </c>
-      <c r="H13">
-        <v>14500000</v>
-      </c>
-      <c r="I13" t="str">
-        <v>14.5M EGP</v>
-      </c>
-      <c r="J13">
-        <v>170</v>
-      </c>
-      <c r="K13">
-        <v>3</v>
-      </c>
-      <c r="L13">
-        <v>2</v>
-      </c>
-      <c r="M13" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N13" t="str">
-        <v>Direct Owner</v>
-      </c>
-      <c r="O13" t="str">
-        <v/>
-      </c>
-      <c r="P13" t="str">
-        <v/>
-      </c>
-      <c r="Q13" t="str">
-        <v>Active</v>
-      </c>
-      <c r="R13" t="str">
-        <v>high-confidence</v>
-      </c>
-      <c r="S13" t="str">
-        <v>https://images.unsplash.com/photo-1600596542815-ffad4c1539a9</v>
-      </c>
-      <c r="T13" t="str">
-        <v>Automated Vitest Verification Unit</v>
-      </c>
-      <c r="U13" t="str">
-        <v>Direct owner</v>
-      </c>
-      <c r="V13" t="str">
-        <v>2026-10-19T04:11:26.991Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1645,7 +965,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V2" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
     <row r="3">
@@ -1713,7 +1033,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V3" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
   </sheetData>
@@ -1860,7 +1180,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V2" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
     <row r="3">
@@ -1928,7 +1248,7 @@
         <v>structural-seed</v>
       </c>
       <c r="V3" t="str">
-        <v>2026-10-19T03:54:03.055Z</v>
+        <v>2026-10-19T04:27:16.073Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>